<commit_message>
Added the required **GRANTs**, the new version of the **APEX application**, and the corresponding changes to the package.
</commit_message>
<xml_diff>
--- a/docs/ADRE_OPS_Table_Inventory.xlsx
+++ b/docs/ADRE_OPS_Table_Inventory.xlsx
@@ -5,17 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JCCC\ArGlobal-1\Create-item-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA2F515F-DFCC-4C5B-8CB4-F85D9D4B87C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CE5856-113F-4C16-8C70-832972574A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15690" yWindow="410" windowWidth="5570" windowHeight="3590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OPS Tables" sheetId="1" r:id="rId1"/>
     <sheet name="SQL Commands" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPS Tables'!$A$4:$E$22</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -508,6 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
@@ -561,7 +565,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" hidden="1">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -578,7 +582,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" hidden="1">
       <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
@@ -595,7 +599,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" hidden="1">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
@@ -612,7 +616,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" hidden="1">
       <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
@@ -629,7 +633,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" hidden="1">
       <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
@@ -646,7 +650,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" hidden="1">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
@@ -663,7 +667,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" hidden="1">
       <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
@@ -833,7 +837,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" hidden="1">
       <c r="A21" s="4" t="s">
         <v>11</v>
       </c>
@@ -850,7 +854,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" hidden="1">
       <c r="A22" s="4" t="s">
         <v>11</v>
       </c>
@@ -868,6 +872,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:E22" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Yes"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>